<commit_message>
Supervisor beheert medewerkers + fix projectensync na Teamleader-accountwissel
</commit_message>
<xml_diff>
--- a/uurivokostprijsecofinity.xlsx
+++ b/uurivokostprijsecofinity.xlsx
@@ -323,10 +323,10 @@
     <t xml:space="preserve">Aanvullend (nieuw): Render workspace-abonnement meegerekend</t>
   </si>
   <si>
-    <t xml:space="preserve">De gratis Render Hobby-workspace volstaat tot 25 services totaal (Aannames!B26). Bij 2 services/klant (Aannames!B28, basisscenario zonder Redis) ligt de drempel dus bij </t>
-  </si>
-  <si>
-    <t xml:space="preserve">klanten — daarna: vlak $25/maand (Aannames!B27), ongeacht hoeveel erboven.</t>
+    <t xml:space="preserve">De gratis Render Hobby-workspace volstaat tot 25 services totaal (Aannames!B26). Bij 2 services/klant (Aannames!B28, basisscenario zonder Redis) blijft dit dus gratis tot en met </t>
+  </si>
+  <si>
+    <t xml:space="preserve">klanten (24 services); vanaf de volgende klant betaal je het vlakke $25/maand-tarief (Aannames!B27), ongeacht hoeveel erboven.</t>
   </si>
   <si>
     <t xml:space="preserve">Render workspace-abonnement (0 tot de grens hierboven, dan vlak tarief)</t>
@@ -2156,7 +2156,7 @@
       <c r="F19" s="41"/>
       <c r="G19" s="41"/>
     </row>
-    <row r="20" customFormat="false" ht="53.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="79.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="42" t="s">
         <v>99</v>
       </c>

</xml_diff>